<commit_message>
fav ico try again
</commit_message>
<xml_diff>
--- a/members.xlsx
+++ b/members.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\ariston\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBF1100D-FDD6-40BE-B0EA-93E6FA977CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2771A5-5940-4280-8DFB-1FCC1645F0FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="72">
   <si>
     <t>Όνομα μέλους</t>
   </si>
@@ -219,6 +219,30 @@
   </si>
   <si>
     <t>kammasofia@yahoo.com</t>
+  </si>
+  <si>
+    <t>Σταύρος</t>
+  </si>
+  <si>
+    <t>stauroskarras@icloud.com</t>
+  </si>
+  <si>
+    <t>antonis</t>
+  </si>
+  <si>
+    <t>cubotkonst@gmail.com</t>
+  </si>
+  <si>
+    <t>ΖΑΧΑΡΗ ΧΡΥΣΟΥΛΑ</t>
+  </si>
+  <si>
+    <t>chryza_samos@hotmail.com</t>
+  </si>
+  <si>
+    <t>ΓΙΩΡΓΟΣ ΧΡΙΣΤΟΔΟΥΛΑΚΗΣ</t>
+  </si>
+  <si>
+    <t>christod@sch.gr</t>
   </si>
 </sst>
 </file>
@@ -1613,13 +1637,21 @@
       <c r="L25" s="6"/>
     </row>
     <row r="26" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>64</v>
+      </c>
       <c r="C26" t="s">
         <v>30</v>
       </c>
+      <c r="D26" s="8">
+        <v>46036</v>
+      </c>
       <c r="E26" t="s">
         <v>55</v>
       </c>
-      <c r="F26" s="6"/>
+      <c r="F26" s="11" t="s">
+        <v>65</v>
+      </c>
       <c r="G26" t="s">
         <v>30</v>
       </c>
@@ -1631,14 +1663,22 @@
       </c>
       <c r="L26" s="6"/>
     </row>
-    <row r="27" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="C27" t="s">
         <v>30</v>
       </c>
+      <c r="D27" s="8">
+        <v>46037</v>
+      </c>
       <c r="E27" t="s">
         <v>55</v>
       </c>
-      <c r="F27" s="6"/>
+      <c r="F27" s="11" t="s">
+        <v>67</v>
+      </c>
       <c r="G27" t="s">
         <v>30</v>
       </c>
@@ -1650,14 +1690,22 @@
       </c>
       <c r="L27" s="6"/>
     </row>
-    <row r="28" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>68</v>
+      </c>
       <c r="C28" t="s">
         <v>30</v>
       </c>
+      <c r="D28" s="8">
+        <v>46038</v>
+      </c>
       <c r="E28" t="s">
         <v>55</v>
       </c>
-      <c r="F28" s="6"/>
+      <c r="F28" s="11" t="s">
+        <v>69</v>
+      </c>
       <c r="G28" t="s">
         <v>30</v>
       </c>
@@ -1670,13 +1718,21 @@
       <c r="L28" s="6"/>
     </row>
     <row r="29" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="C29" t="s">
         <v>30</v>
       </c>
+      <c r="D29" s="8">
+        <v>46038</v>
+      </c>
       <c r="E29" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="6"/>
+      <c r="F29" s="10" t="s">
+        <v>71</v>
+      </c>
       <c r="G29" t="s">
         <v>30</v>
       </c>
@@ -4978,15 +5034,19 @@
     <hyperlink ref="A23" r:id="rId20" display="https://aristonwashdry.gr/admin/users/22" xr:uid="{424361F0-C923-4090-B22A-8D929733C462}"/>
     <hyperlink ref="A24" r:id="rId21" display="https://aristonwashdry.gr/admin/users/23" xr:uid="{2B0BBC98-57C8-4B3A-9FD0-B376E28BDB15}"/>
     <hyperlink ref="A25" r:id="rId22" display="https://aristonwashdry.gr/admin/users/24" xr:uid="{1EA05C9D-D2C1-4E32-B83A-076353DAF0E0}"/>
+    <hyperlink ref="A26" r:id="rId23" display="https://aristonwashdry.gr/admin/users/25" xr:uid="{E037CB8A-369A-41BA-9375-D58657095ECF}"/>
+    <hyperlink ref="A27" r:id="rId24" display="https://aristonwashdry.gr/admin/users/26" xr:uid="{9A63AA3C-6810-4DDC-A6F9-4124CB764198}"/>
+    <hyperlink ref="A28" r:id="rId25" display="https://aristonwashdry.gr/admin/users/27" xr:uid="{2E7B9671-EBCD-43FC-9F81-743195FAA25B}"/>
+    <hyperlink ref="A29" r:id="rId26" display="https://aristonwashdry.gr/admin/users/28" xr:uid="{3B9F3F50-80F2-48C5-B49E-23F0B2CF39BF}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="48" fitToHeight="0" orientation="landscape" r:id="rId23"/>
+  <pageSetup scale="48" fitToHeight="0" orientation="landscape" r:id="rId27"/>
   <headerFooter differentFirst="1">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId24"/>
+    <tablePart r:id="rId28"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>